<commit_message>
Add Chugoku region (Tottori/Shimane/Okayama/Hiroshima/Yamaguchi) hospital Excels
Fix category classification bug: items named like "回診用X線撮影装置"
were mis-labeled as 一般撮影（レントゲン） because the generic keyword
"X線撮影装置" was checked before the more specific 回診用 category.
Reordered CATEGORIES so 回診用X線装置 is checked first, and relabeled
the affected rows in previously delivered hospital/regional files
(みなと, 和歌山, 京都第二, 芳賀, 静岡, 松江).
</commit_message>
<xml_diff>
--- a/output/京都第二赤十字病院_随意契約_X線関連.xlsx
+++ b/output/京都第二赤十字病院_随意契約_X線関連.xlsx
@@ -561,7 +561,7 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>一般撮影（レントゲン）</t>
+          <t>回診用X線装置</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
@@ -659,7 +659,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>一般撮影（レントゲン）</t>
+          <t>回診用X線装置</t>
         </is>
       </c>
       <c r="B4" s="3" t="n">
@@ -670,7 +670,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>透視撮影台（X線テレビ）</t>
+          <t>一般撮影（レントゲン）</t>
         </is>
       </c>
       <c r="B5" s="3" t="n">
@@ -685,33 +685,33 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>血管撮影（CVS、アンギオ）</t>
+          <t>透視撮影台（X線テレビ）</t>
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C6" s="3" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>公表された随意契約に該当なし</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>外科用イメージ（可搬型Cアーム透視装置）</t>
+          <t>血管撮影（CVS、アンギオ）</t>
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>公表された随意契約に該当なし</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>回診用X線装置</t>
+          <t>外科用イメージ（可搬型Cアーム透視装置）</t>
         </is>
       </c>
       <c r="B8" s="3" t="n">

</xml_diff>